<commit_message>
Fix Bug Name Stock Upper Case & Lower Case
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -1,37 +1,147 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StockInvestment\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B92C35-E9E8-400B-9C7C-EE94ED43978C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="4260" yWindow="4635" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Avg_Price</t>
+  </si>
+  <si>
+    <t>PTT</t>
+  </si>
+  <si>
+    <t>CPALL</t>
+  </si>
+  <si>
+    <t>GFPT</t>
+  </si>
+  <si>
+    <t>NSL</t>
+  </si>
+  <si>
+    <t>SORKON</t>
+  </si>
+  <si>
+    <t>ACE</t>
+  </si>
+  <si>
+    <t>BCP</t>
+  </si>
+  <si>
+    <t>TTW</t>
+  </si>
+  <si>
+    <t>BAM</t>
+  </si>
+  <si>
+    <t>TIDLOR</t>
+  </si>
+  <si>
+    <t>TQM</t>
+  </si>
+  <si>
+    <t>DMT</t>
+  </si>
+  <si>
+    <t>KEX</t>
+  </si>
+  <si>
+    <t>PRM</t>
+  </si>
+  <si>
+    <t>STGT</t>
+  </si>
+  <si>
+    <t>LPN</t>
+  </si>
+  <si>
+    <t>QH</t>
+  </si>
+  <si>
+    <t>CPAXT</t>
+  </si>
+  <si>
+    <t>CPF</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
+    <t>PTTEP</t>
+  </si>
+  <si>
+    <t>RATCH</t>
+  </si>
+  <si>
+    <t>KTB</t>
+  </si>
+  <si>
+    <t>BDMS</t>
+  </si>
+  <si>
+    <t>BEM</t>
+  </si>
+  <si>
+    <t>BTS</t>
+  </si>
+  <si>
+    <t>CRC</t>
+  </si>
+  <si>
+    <t>LH</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +156,46 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,68 +483,338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Symbol</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Avg_Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>PTT</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>300</v>
+      </c>
+      <c r="C2">
+        <v>10.52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <v>13.02</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>100</v>
+      </c>
+      <c r="C4">
+        <v>4.6500000000000004</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>1960</v>
+      </c>
+      <c r="C5">
+        <v>4.83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1500</v>
+      </c>
+      <c r="C6">
+        <v>2.94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>100</v>
+      </c>
+      <c r="C7">
+        <v>14.52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1100</v>
+      </c>
+      <c r="C8">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>500</v>
+      </c>
+      <c r="C9">
+        <v>16.190000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>627</v>
+      </c>
+      <c r="C10">
+        <v>27.32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>200</v>
+      </c>
+      <c r="C11">
+        <v>38.94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
         <v>1000</v>
       </c>
-      <c r="C2" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CPALL</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+      <c r="C12">
+        <v>12.39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>1200</v>
+      </c>
+      <c r="C13">
+        <v>22.85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>100</v>
+      </c>
+      <c r="C14">
+        <v>5.51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>2100</v>
+      </c>
+      <c r="C15">
+        <v>23.27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>100</v>
+      </c>
+      <c r="C16">
+        <v>3.81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>200</v>
+      </c>
+      <c r="C17">
+        <v>2.0699999999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18">
+        <v>394</v>
+      </c>
+      <c r="C18">
+        <v>42.61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19">
+        <v>1400</v>
+      </c>
+      <c r="C19">
+        <v>24.37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20">
+        <v>1900</v>
+      </c>
+      <c r="C20">
+        <v>23.54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21">
+        <v>200</v>
+      </c>
+      <c r="C21">
+        <v>27.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22">
+        <v>200</v>
+      </c>
+      <c r="C22">
+        <v>70.489999999999995</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23">
+        <v>1000</v>
+      </c>
+      <c r="C23">
+        <v>43.75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24">
+        <v>1000</v>
+      </c>
+      <c r="C24">
+        <v>10.199999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25">
+        <v>600</v>
+      </c>
+      <c r="C25">
+        <v>20.18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26">
+        <v>200</v>
+      </c>
+      <c r="C26">
+        <v>7.64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27">
         <v>500</v>
       </c>
-      <c r="C3" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DELTA</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+      <c r="C27">
+        <v>8.17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28">
         <v>100</v>
       </c>
-      <c r="C4" t="n">
-        <v>100</v>
+      <c r="C28">
+        <v>53.84</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29">
+        <v>200</v>
+      </c>
+      <c r="C29">
+        <v>25.42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>400</v>
+      </c>
+      <c r="C30">
+        <v>7.24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>